<commit_message>
Data sync: 72 words · 200 phrases · 0 new images
</commit_message>
<xml_diff>
--- a/update_data_folder/WordList.xlsx
+++ b/update_data_folder/WordList.xlsx
@@ -6646,47 +6646,47 @@
         <v>vocab-food</v>
       </c>
       <c r="B2" t="str">
-        <v>mushroom</v>
+        <v>beef</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>vocab-places</v>
+        <v>vocab-animal</v>
       </c>
       <c r="B3" t="str">
-        <v>airport</v>
+        <v>bird</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>vocab-animal</v>
+        <v>vocab-body</v>
       </c>
       <c r="B4" t="str">
-        <v>pig</v>
+        <v>hand</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>vocab-body</v>
+        <v>vocab-clothes</v>
       </c>
       <c r="B5" t="str">
-        <v>eye</v>
+        <v>hat</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>vocab-clothes</v>
+        <v>vocab-colors</v>
       </c>
       <c r="B6" t="str">
-        <v>pants</v>
+        <v>pink</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>vocab-colors</v>
+        <v>vocab-places</v>
       </c>
       <c r="B7" t="str">
-        <v>yellow</v>
+        <v>bank</v>
       </c>
     </row>
     <row r="8">
@@ -6694,31 +6694,31 @@
         <v>oral-everyday</v>
       </c>
       <c r="B8" t="str">
-        <v>orange</v>
+        <v>cake</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>oral-opinions</v>
+        <v>oral-food</v>
       </c>
       <c r="B9" t="str">
-        <v>cherry</v>
+        <v>beef</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>oral-food</v>
+        <v>oral-emotions</v>
       </c>
       <c r="B10" t="str">
-        <v>hungry</v>
+        <v>bear</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>oral-emotions</v>
+        <v>oral-opinions</v>
       </c>
       <c r="B11" t="str">
-        <v>durian</v>
+        <v>elephant</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data sync: 158 words · 200 phrases · 89 new images
</commit_message>
<xml_diff>
--- a/update_data_folder/WordList.xlsx
+++ b/update_data_folder/WordList.xlsx
@@ -729,7 +729,7 @@
         <v>Animals</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" t="str">
         <v>海鸥</v>
@@ -799,7 +799,7 @@
         <v>Food</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" t="str">
         <v>榴莲</v>
@@ -1427,7 +1427,7 @@
         <v>Food</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" t="str">
         <v>西兰花</v>
@@ -2111,7 +2111,7 @@
         <v>Body</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F47" t="str">
         <v>骷髅</v>
@@ -2377,7 +2377,7 @@
         <v>Clothes</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F54" t="str">
         <v>凉鞋</v>
@@ -2675,7 +2675,7 @@
         <v>Purple Cabbage is wearing too many layers and can't take them off!</v>
       </c>
       <c r="C62" t="str">
-        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round purple cabbage with a frustrated face, wrapped in many ruffled leafy layers bulging outward"</v>
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round purple cabbage with a frustrated face, wrapped in many ruffled leafy layers bulging outward, purely purple color"</v>
       </c>
       <c r="D62" t="str">
         <v>Colors</v>
@@ -2751,7 +2751,7 @@
         <v>White Snowman is eating an ice pop to stay cool!</v>
       </c>
       <c r="C64" t="str">
-        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round white snowman with a happy relaxed face, wearing a top hat and a tiny striped scarf, holding a blue ice pop"</v>
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round white snowman with a happy relaxed face, wearing a top hat and a tiny striped scarf, holding a blue ice pop, no legs no foot"</v>
       </c>
       <c r="D64" t="str">
         <v>Colors</v>
@@ -3321,7 +3321,7 @@
         <v>Ice Cream is crowning herself queen with her cone hat!</v>
       </c>
       <c r="C79" t="str">
-        <v>PlushStyle, plush style, high resolution, rich and elaborate details, white background, a super cute plush toy of "a pink ice cream with a smug smile, lifting her waffle cone like a royal crown"</v>
+        <v>PlushStyle, plush style, high resolution, rich and elaborate details, white background, a super cute plush toy of "a pink ice cream with a smug queenly face, placing her upside-down waffle cone on top like a crown"</v>
       </c>
       <c r="D79" t="str">
         <v>Food</v>
@@ -3707,7 +3707,7 @@
         <v>Food</v>
       </c>
       <c r="E89">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F89" t="str">
         <v>海藻</v>
@@ -3777,7 +3777,7 @@
         <v>Soup is hiding from the big scary spoon!</v>
       </c>
       <c r="C91" t="str">
-        <v>PlushStyle, plush style, high resolution, rich and elaborate details, white background, a super cute plush toy of "a small soup bowl with a panicked face, hiding behind a napkin, a large spoon looming close"</v>
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a small soup bowl with a frightened face peeking out, a large spoon looming over it"</v>
       </c>
       <c r="D91" t="str">
         <v>Food</v>
@@ -3812,7 +3812,10 @@
         <v>steak</v>
       </c>
       <c r="B92" t="str">
-        <v>Steak is flexing his juicy muscles on the plate!</v>
+        <v>The steak feels so cozy wrapped in its pastry blanket — beef Wellington style.</v>
+      </c>
+      <c r="C92" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a thick steak snugly wrapped in a golden pastry crust like a blanket, with a cozy sleepy smile"</v>
       </c>
       <c r="D92" t="str">
         <v>Food</v>
@@ -3847,7 +3850,10 @@
         <v>sunflower</v>
       </c>
       <c r="B93" t="str">
-        <v>Sunflower has a sore neck from her giant heavy head!</v>
+        <v>The sunflower has a stiff neck from staring at the sun all day.</v>
+      </c>
+      <c r="C93" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a tall sunflower tilting its big flower head to one side with a tired face, a tiny bright sun in the corner"</v>
       </c>
       <c r="D93" t="str">
         <v>Food</v>
@@ -3882,7 +3888,10 @@
         <v>tea</v>
       </c>
       <c r="B94" t="str">
-        <v>Tea is splashing in her hot tub with a teabag floaty!</v>
+        <v>The tea bag starts spilling all the gossip the moment it hits hot water.</v>
+      </c>
+      <c r="C94" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a tea bag sitting in a small cup of light green tea with a chatty excited face, a speech bubble with '!' next to it, having little cute feet"</v>
       </c>
       <c r="D94" t="str">
         <v>Food</v>
@@ -3917,7 +3926,10 @@
         <v>tomato</v>
       </c>
       <c r="B95" t="str">
-        <v>Tomato is sneaking into the fruit club in a fake mustache.</v>
+        <v>The tomato turns even redder when it's embarrassed.</v>
+      </c>
+      <c r="C95" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round deep-red tomato covering its cheeks with tiny hands, with a shy blushing face"</v>
       </c>
       <c r="D95" t="str">
         <v>Food</v>
@@ -3952,7 +3964,10 @@
         <v>water</v>
       </c>
       <c r="B96" t="str">
-        <v>Water spills herself on purpose just to steal the spotlight.</v>
+        <v>The water can never keep a secret — it's completely see-through.</v>
+      </c>
+      <c r="C96" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a tall clear glass of water with a nervous embarrassed face, a tiny key visible inside its transparent body"</v>
       </c>
       <c r="D96" t="str">
         <v>Food</v>
@@ -3987,7 +4002,10 @@
         <v>bag</v>
       </c>
       <c r="B97" t="str">
-        <v>Bag swallowed the keys again and is playing dumb.</v>
+        <v>The bag ate too much and now the zipper won't close.</v>
+      </c>
+      <c r="C97" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round overstuffed backpack with a bursting open zipper, with a guilty satisfied face"</v>
       </c>
       <c r="D97" t="str">
         <v>Items</v>
@@ -4022,7 +4040,10 @@
         <v>bed</v>
       </c>
       <c r="B98" t="str">
-        <v>Bed is giving the warmest hug in the whole house.</v>
+        <v>The bed is so sleepy — everyone naps on it but nobody lets it rest.</v>
+      </c>
+      <c r="C98" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a small bed with half-closed drowsy eyes on the headboard, a sleepy yawning face, ZZZ floating above"</v>
       </c>
       <c r="D98" t="str">
         <v>Items</v>
@@ -4057,7 +4078,10 @@
         <v>book</v>
       </c>
       <c r="B99" t="str">
-        <v>Book keeps dozing off and closing herself mid-story.</v>
+        <v>The book is so thick it's out of breath halfway through.</v>
+      </c>
+      <c r="C99" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a very thick closed book with a bookmark poking out halfway, with an exhausted panting face on the cover and tiny sweat drops"</v>
       </c>
       <c r="D99" t="str">
         <v>Items</v>
@@ -4092,7 +4116,10 @@
         <v>bowl</v>
       </c>
       <c r="B100" t="str">
-        <v>Bowl is slurping up his own soup when nobody's looking!</v>
+        <v>The bowl thinks it's a swimming pool every time it's filled with soup.</v>
+      </c>
+      <c r="C100" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round blue bowl wearing tiny sunglasses with a chill face, a few small vegetables floating in light yellow soup like swimmers, having little cute feet"</v>
       </c>
       <c r="D100" t="str">
         <v>Items</v>
@@ -4129,11 +4156,14 @@
       <c r="B101" t="str">
         <v>Calculator is judging everyone's math with a smug little face.</v>
       </c>
+      <c r="C101" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a calculator with a smug face, chin slightly raised, eyes half-closed in a judging look"</v>
+      </c>
       <c r="D101" t="str">
         <v>Items</v>
       </c>
       <c r="E101">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F101" t="str">
         <v>计算器</v>
@@ -4164,6 +4194,9 @@
       <c r="B102" t="str">
         <v>Camera keeps taking selfies with her own flash!</v>
       </c>
+      <c r="C102" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a camera with its flash popping bright, holding a tiny mirror with a dazzled grinning face"</v>
+      </c>
       <c r="D102" t="str">
         <v>Items</v>
       </c>
@@ -4199,6 +4232,9 @@
       <c r="B103" t="str">
         <v>Chair is SO tired of holding everyone's heavy bottoms!</v>
       </c>
+      <c r="C103" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a wooden chair with shaky wobbly legs, with an exhausted annoyed face and tiny sweat drops"</v>
+      </c>
       <c r="D103" t="str">
         <v>Items</v>
       </c>
@@ -4234,6 +4270,9 @@
       <c r="B104" t="str">
         <v>Charger is giving his phone friend a big energy hug!</v>
       </c>
+      <c r="C104" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a charger cable wrapping around a small phone like a hug, both with happy smiling faces"</v>
+      </c>
       <c r="D104" t="str">
         <v>Items</v>
       </c>
@@ -4269,6 +4308,9 @@
       <c r="B105" t="str">
         <v>Computer has 47 tabs open and a splitting headache!</v>
       </c>
+      <c r="C105" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a laptop with many tiny tabs popping out of the screen, with a pained headache face and a small ice pack on top"</v>
+      </c>
       <c r="D105" t="str">
         <v>Items</v>
       </c>
@@ -4304,6 +4346,9 @@
       <c r="B106" t="str">
         <v>Cup is holding her breath so the water won't spill!</v>
       </c>
+      <c r="C106" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a cup filled to the very brim with water, puffing its cheeks with a nervous tense face"</v>
+      </c>
       <c r="D106" t="str">
         <v>Items</v>
       </c>
@@ -4339,6 +4384,9 @@
       <c r="B107" t="str">
         <v>Door is sick of being slammed and wants an apology!</v>
       </c>
+      <c r="C107" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a wooden door with an angry pouty face, one small arm crossed, a red bump mark on its edge"</v>
+      </c>
       <c r="D107" t="str">
         <v>Items</v>
       </c>
@@ -4374,6 +4422,9 @@
       <c r="B108" t="str">
         <v>Fork is poking everything just to say hi!</v>
       </c>
+      <c r="C108" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a silver fork with a cheerful eager face, poking a tiny round tomato with its prongs"</v>
+      </c>
       <c r="D108" t="str">
         <v>Items</v>
       </c>
@@ -4409,6 +4460,9 @@
       <c r="B109" t="str">
         <v>Headphones are whispering secrets straight into your ears!</v>
       </c>
+      <c r="C109" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a pair of headphones with a mischievous whispering face, a tiny speech bubble with '🤫' between the ear cups"</v>
+      </c>
       <c r="D109" t="str">
         <v>Items</v>
       </c>
@@ -4444,6 +4498,9 @@
       <c r="B110" t="str">
         <v>Key thinks every lock is a puzzle only she can solve.</v>
       </c>
+      <c r="C110" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a detective-style golden key with a confident smirk, standing next to a small padlock with a puzzled face"</v>
+      </c>
       <c r="D110" t="str">
         <v>Items</v>
       </c>
@@ -4479,6 +4536,9 @@
       <c r="B111" t="str">
         <v>Knife is bragging about being the sharpest one in the drawer!</v>
       </c>
+      <c r="C111" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a shiny kitchen knife with a proud smirk and chin raised, standing on a small open drawer"</v>
+      </c>
       <c r="D111" t="str">
         <v>Items</v>
       </c>
@@ -4514,6 +4574,9 @@
       <c r="B112" t="str">
         <v>Laptop is burning up from binge-watching cat videos all night!</v>
       </c>
+      <c r="C112" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a laptop with a red overheated face, a tiny cat icon on its screen, small heat waves rising from the top"</v>
+      </c>
       <c r="D112" t="str">
         <v>Items</v>
       </c>
@@ -4546,6 +4609,9 @@
       <c r="B113" t="str">
         <v>Map is lost and too embarrassed to ask for directions!</v>
       </c>
+      <c r="C113" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a folded map with colorful route lines on it, held upside-down with a confused embarrassed face, tiny sweat drops and a '?' above"</v>
+      </c>
       <c r="D113" t="str">
         <v>Items</v>
       </c>
@@ -4566,6 +4632,9 @@
       </c>
       <c r="J113" t="str">
         <v>/mæp/</v>
+      </c>
+      <c r="K113" t="str">
+        <v>地图自己迷路了，还不好意思开口问路！</v>
       </c>
       <c r="L113" t="str">
         <v>ちずくんがまいごになっちゃったの。でも、ひとにみちをきくのがはずかしくて、じっとしてるんだって。</v>
@@ -4578,6 +4647,9 @@
       <c r="B114" t="str">
         <v>Money is hiding in the couch cushions for a secret vacation!</v>
       </c>
+      <c r="C114" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a green dollar bill with sunglasses and a relaxed happy face, hiding inside a small sofa gap"</v>
+      </c>
       <c r="D114" t="str">
         <v>Items</v>
       </c>
@@ -4598,6 +4670,9 @@
       </c>
       <c r="J114" t="str">
         <v>/ˈmʌni/</v>
+      </c>
+      <c r="K114" t="str">
+        <v>钞票偷偷躲在沙发垫里，计划一场秘密度假！</v>
       </c>
       <c r="L114" t="str">
         <v>おかねちゃんがソファーのすきまにかくれて、ないしょのばかんすをしてるの。</v>
@@ -4610,6 +4685,9 @@
       <c r="B115" t="str">
         <v>Phone keeps pocket-dialing everyone and blaming the pants.</v>
       </c>
+      <c r="C115" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a phone with a cheeky innocent face poking out of a jeans pocket, the pocket with an annoyed face"</v>
+      </c>
       <c r="D115" t="str">
         <v>Items</v>
       </c>
@@ -4630,6 +4708,9 @@
       </c>
       <c r="J115" t="str">
         <v>/foʊn/</v>
+      </c>
+      <c r="K115" t="str">
+        <v>手机总误拨电话给所有人，还赖是裤子的锅。</v>
       </c>
       <c r="L115" t="str">
         <v>けいたいくんがポケットのなかでだれかにかけちゃって、それをズボンのせいにしてるんだ。</v>
@@ -4642,6 +4723,9 @@
       <c r="B116" t="str">
         <v>Plate is showing off her fancy gold rim like a new necklace.</v>
       </c>
+      <c r="C116" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round white plate with a shiny gold rim, with a proud glamorous face, tilting slightly to show off the rim"</v>
+      </c>
       <c r="D116" t="str">
         <v>Items</v>
       </c>
@@ -4662,6 +4746,9 @@
       </c>
       <c r="J116" t="str">
         <v>/pleɪt/</v>
+      </c>
+      <c r="K116" t="str">
+        <v>盘子炫耀自己漂亮的金边，像戴了条新项链。</v>
       </c>
       <c r="L116" t="str">
         <v>おさらちゃんがきれいなきんのふちを、あたらしいネックレスみたいにみせびらかしてるの。</v>
@@ -4674,6 +4761,9 @@
       <c r="B117" t="str">
         <v>Saw keeps falling asleep mid-cut and snoring "zzzzzz"!</v>
       </c>
+      <c r="C117" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a handsaw resting on a half-cut piece of wood, with closed sleepy eyes and ZZZ floating above"</v>
+      </c>
       <c r="D117" t="str">
         <v>Items</v>
       </c>
@@ -4694,6 +4784,9 @@
       </c>
       <c r="J117" t="str">
         <v>/sɔː/</v>
+      </c>
+      <c r="K117" t="str">
+        <v>锯子锯到一半就睡着，还打起了呼噜！</v>
       </c>
       <c r="L117" t="str">
         <v>のこぎりくんがきりかけでねむっちゃって、「すーすー」ないてるんだ。</v>
@@ -4706,6 +4799,9 @@
       <c r="B118" t="str">
         <v>Scale is lying about everyone's weight just to make friends.</v>
       </c>
+      <c r="C118" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a bathroom scale with a sneaky winking face, its display showing a tiny number with a speech bubble '😉'"</v>
+      </c>
       <c r="D118" t="str">
         <v>Items</v>
       </c>
@@ -4726,6 +4822,9 @@
       </c>
       <c r="J118" t="str">
         <v>/skeɪl/</v>
+      </c>
+      <c r="K118" t="str">
+        <v>体重秤为了交朋友，对每个人的体重都撒了谎。</v>
       </c>
       <c r="L118" t="str">
         <v>たいじょうけいくんがみんなのたいじゅうをうそついて、ともだちをつくろうとしてるの。</v>
@@ -4738,6 +4837,9 @@
       <c r="B119" t="str">
         <v>Scarecrow is posing all day and calling it "modeling."</v>
       </c>
+      <c r="C119" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a scarecrow with a fashionable confident face, one arm out in a model pose, wearing a tiny straw hat"</v>
+      </c>
       <c r="D119" t="str">
         <v>Items</v>
       </c>
@@ -4758,6 +4860,9 @@
       </c>
       <c r="J119" t="str">
         <v>/ˈskɛrkroʊ/</v>
+      </c>
+      <c r="K119" t="str">
+        <v>稻草人整天摆姿势，还管这叫"走台步"。</v>
       </c>
       <c r="L119" t="str">
         <v>かかしさんがいちにちじゅうポーズをとって、それを「モデル」のしごとだっておもってるんだって。</v>
@@ -4770,6 +4875,9 @@
       <c r="B120" t="str">
         <v>Scissors only get things done when they finally shut up!</v>
       </c>
+      <c r="C120" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a pair of scissors with a smug satisfied face on the handle, blades closed tight, snipping a piece of paper"</v>
+      </c>
       <c r="D120" t="str">
         <v>Items</v>
       </c>
@@ -4790,6 +4898,9 @@
       </c>
       <c r="J120" t="str">
         <v>/ˈsɪzərz/</v>
+      </c>
+      <c r="K120" t="str">
+        <v>剪刀只有闭上嘴，才能真正办成事！</v>
       </c>
       <c r="L120" t="str">
         <v>はさみくんはやっとおしゃべりをやめたときに、やっとしごとができるんだって。</v>
@@ -4802,11 +4913,14 @@
       <c r="B121" t="str">
         <v>Screwdriver thinks every problem just needs one more twist.</v>
       </c>
+      <c r="C121" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a screwdriver with a determined confident face, pressing down on a tiny screw with a speech bubble '1 more!'"</v>
+      </c>
       <c r="D121" t="str">
         <v>Items</v>
       </c>
       <c r="E121">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F121" t="str">
         <v>螺丝刀</v>
@@ -4822,6 +4936,9 @@
       </c>
       <c r="J121" t="str">
         <v>/ˈskruːˌdraɪvər/</v>
+      </c>
+      <c r="K121" t="str">
+        <v>螺丝刀觉得所有问题都只需要再拧一下。</v>
       </c>
       <c r="L121" t="str">
         <v>ねじまわしくんは、どんなこまったことも、もういっかいまげばなんとかなるっておもってるの。</v>
@@ -4834,6 +4951,9 @@
       <c r="B122" t="str">
         <v>Shell carries her house everywhere, just in case she needs a nap!</v>
       </c>
+      <c r="C122" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a fancily accessorized seashell half-open like a bed, with a cozy sleepy face peeking out, ZZZ floating above"</v>
+      </c>
       <c r="D122" t="str">
         <v>Items</v>
       </c>
@@ -4869,6 +4989,9 @@
       <c r="B123" t="str">
         <v>Shield never peeks at what's flying toward him!</v>
       </c>
+      <c r="C123" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a round metal shield with eyes squeezed shut and a scared face, a tiny arrow stuck on its surface"</v>
+      </c>
       <c r="D123" t="str">
         <v>Items</v>
       </c>
@@ -4904,6 +5027,9 @@
       <c r="B124" t="str">
         <v>Shovel keeps digging up secrets nobody asked for!</v>
       </c>
+      <c r="C124" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a shovel with a mischievous gossipy face, digging into a small dirt pile with a speech bubble '👀'"</v>
+      </c>
       <c r="D124" t="str">
         <v>Items</v>
       </c>
@@ -4939,6 +5065,9 @@
       <c r="B125" t="str">
         <v>Sock ran away from the laundry to live a single life!</v>
       </c>
+      <c r="C125" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a single colorful sock with a happy free-spirited face, wearing tiny sunglasses, both small arms raised in a cheerful wave"</v>
+      </c>
       <c r="D125" t="str">
         <v>Items</v>
       </c>
@@ -4974,6 +5103,9 @@
       <c r="B126" t="str">
         <v>Sofa has swallowed three remotes and isn't giving them back!</v>
       </c>
+      <c r="C126" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a plump sofa with a cheeky grinning face, three remote corners poking out between its cushions"</v>
+      </c>
       <c r="D126" t="str">
         <v>Items</v>
       </c>
@@ -5009,6 +5141,9 @@
       <c r="B127" t="str">
         <v>Spoon is jealous that Fork gets all the fun poking jobs!</v>
       </c>
+      <c r="C127" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a spoon with a jealous pouty face, watching a small fork happily poking a tiny piece of food"</v>
+      </c>
       <c r="D127" t="str">
         <v>Items</v>
       </c>
@@ -5044,6 +5179,9 @@
       <c r="B128" t="str">
         <v>Stethoscope is eavesdropping on everyone's heartbeat gossip!</v>
       </c>
+      <c r="C128" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a stethoscope with a nosy eager face on the chest piece, leaning against a tiny red heart with a surprised face"</v>
+      </c>
       <c r="D128" t="str">
         <v>Items</v>
       </c>
@@ -5079,6 +5217,9 @@
       <c r="B129" t="str">
         <v>Suitcase ate too many clothes and can't zip up!</v>
       </c>
+      <c r="C129" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "an overstuffed suitcase with a zipper bursting open, clothes peeking out, with a guilty bloated face"</v>
+      </c>
       <c r="D129" t="str">
         <v>Items</v>
       </c>
@@ -5101,7 +5242,7 @@
         <v>/ˈsuːtkeɪs/</v>
       </c>
       <c r="K129" t="str">
-        <v>行李箱衣服吃撑了，拉链都拉不上啦！</v>
+        <v>行李箱衣服吃撑了，拉链都拉不上了！</v>
       </c>
       <c r="L129" t="str">
         <v>スーツケースくんがふくをたべすぎて、チャックがしまらないんだって！</v>
@@ -5114,6 +5255,9 @@
       <c r="B130" t="str">
         <v>Table is wobbling her bad leg for attention again!</v>
       </c>
+      <c r="C130" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a small wooden table with one shorter wobbly leg, with a dramatic whiny face, tilting to one side"</v>
+      </c>
       <c r="D130" t="str">
         <v>Items</v>
       </c>
@@ -5149,6 +5293,9 @@
       <c r="B131" t="str">
         <v>Telescope is stretching his long neck to spy on the moon.</v>
       </c>
+      <c r="C131" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a detective-style telescope with its tube stretched out long, with a nosy curious face, a tiny moon in the corner"</v>
+      </c>
       <c r="D131" t="str">
         <v>Items</v>
       </c>
@@ -5184,6 +5331,9 @@
       <c r="B132" t="str">
         <v>Tent is holding his breath so he won't collapse!</v>
       </c>
+      <c r="C132" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a green triangular tent puffing its cheeks hard with a tense nervous face, slightly inflated, having little cute feet"</v>
+      </c>
       <c r="D132" t="str">
         <v>Items</v>
       </c>
@@ -5219,6 +5369,9 @@
       <c r="B133" t="str">
         <v>Throne refuses to let anyone sit without a royal appointment!</v>
       </c>
+      <c r="C133" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a Victorian-style golden throne with a snooty proud face, one small arm raised in a 'stop' gesture"</v>
+      </c>
       <c r="D133" t="str">
         <v>Items</v>
       </c>
@@ -5254,6 +5407,9 @@
       <c r="B134" t="str">
         <v>Ticket is terrified of getting ripped in half on his big day!</v>
       </c>
+      <c r="C134" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a colorful ticket with a sad worried face, a tiny dotted tear-line across its middle, trembling with sweat drops, having little cute feet"</v>
+      </c>
       <c r="D134" t="str">
         <v>Items</v>
       </c>
@@ -5289,6 +5445,9 @@
       <c r="B135" t="str">
         <v>Toaster keeps scaring himself every time the bread pops out!</v>
       </c>
+      <c r="C135" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a toaster with a shocked startled face, a piece of toast popping out of the top, having little cute feet"</v>
+      </c>
       <c r="D135" t="str">
         <v>Items</v>
       </c>
@@ -5324,6 +5483,9 @@
       <c r="B136" t="str">
         <v>Toothbrush thinks her messy bristles are a punk hairstyle!</v>
       </c>
+      <c r="C136" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a punk-style toothbrush with wild spiky bristles sticking out in all directions, with a proud cool face"</v>
+      </c>
       <c r="D136" t="str">
         <v>Items</v>
       </c>
@@ -5359,6 +5521,9 @@
       <c r="B137" t="str">
         <v>Trophy won't stop polishing himself for the perfect shine!</v>
       </c>
+      <c r="C137" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a shiny golden trophy holding a tiny cloth, polishing itself with a vain satisfied face, having little cute feet"</v>
+      </c>
       <c r="D137" t="str">
         <v>Items</v>
       </c>
@@ -5394,6 +5559,9 @@
       <c r="B138" t="str">
         <v>TV is mad nobody looks her in the eye anymore — just phones!</v>
       </c>
+      <c r="C138" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a retro-style TV with an angry jealous face on the screen, a tiny smartphone next to it getting all the attention, having little cute feet"</v>
+      </c>
       <c r="D138" t="str">
         <v>Items</v>
       </c>
@@ -5429,6 +5597,9 @@
       <c r="B139" t="str">
         <v>Umbrella is sulking in the corner waiting for a rainy day!</v>
       </c>
+      <c r="C139" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a floral-pattern umbrella with a lonely pouty face, a tiny thought bubble with a rain cloud"</v>
+      </c>
       <c r="D139" t="str">
         <v>Items</v>
       </c>
@@ -5464,6 +5635,9 @@
       <c r="B140" t="str">
         <v>Wallet is on a diet because no money ever comes in!</v>
       </c>
+      <c r="C140" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a very flat thin wallet with a sad hungry face, a tiny belt tightened around it, having little cute feet"</v>
+      </c>
       <c r="D140" t="str">
         <v>Items</v>
       </c>
@@ -5499,6 +5673,9 @@
       <c r="B141" t="str">
         <v>Watering Can has a runny nose that won't stop dripping!</v>
       </c>
+      <c r="C141" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a green watering can with a runny dripping spout, with a sniffly uncomfortable face, having little cute feet"</v>
+      </c>
       <c r="D141" t="str">
         <v>Items</v>
       </c>
@@ -5534,6 +5711,9 @@
       <c r="B142" t="str">
         <v>Window is tired of people only looking through her, never at her!</v>
       </c>
+      <c r="C142" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a Victorian-style window with a sad neglected face on the glass pane, tiny arms crossed with a pouty look"</v>
+      </c>
       <c r="D142" t="str">
         <v>Items</v>
       </c>
@@ -5569,6 +5749,9 @@
       <c r="B143" t="str">
         <v>Cloud is shape-shifting into a bunny to get more likes!</v>
       </c>
+      <c r="C143" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a fluffy white cloud shaped like a bunny with cloud-shaped ears, with a pleased hopeful face, tiny heart-shaped likes floating around"</v>
+      </c>
       <c r="D143" t="str">
         <v>Nature</v>
       </c>
@@ -5604,6 +5787,9 @@
       <c r="B144" t="str">
         <v>Rain keeps knocking on the window but nobody lets him in!</v>
       </c>
+      <c r="C144" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a blue raindrop with a sad pleading face, behind a small window, having little cute feet"</v>
+      </c>
       <c r="D144" t="str">
         <v>Nature</v>
       </c>
@@ -5639,6 +5825,9 @@
       <c r="B145" t="str">
         <v>Snow is an artist, painting everything white.</v>
       </c>
+      <c r="C145" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "an artist-style round snowball holding a paintbrush dripping white paint, with a proud creative face, having little cute feet"</v>
+      </c>
       <c r="D145" t="str">
         <v>Nature</v>
       </c>
@@ -5674,6 +5863,9 @@
       <c r="B146" t="str">
         <v>Snowflake insists she looks nothing like her billion sisters!</v>
       </c>
+      <c r="C146" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a sparkly snowflake with a sassy confident face, next to two identical smaller snowflakes with confused faces, having little cute feet"</v>
+      </c>
       <c r="D146" t="str">
         <v>Nature</v>
       </c>
@@ -5709,6 +5901,9 @@
       <c r="B147" t="str">
         <v>Sun forgot his sunglasses and is squinting at everyone!</v>
       </c>
+      <c r="C147" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a bright yellow sun with squinting eyes and a bothered face, sunglasses sitting on top of its head forgotten, having little cute feet"</v>
+      </c>
       <c r="D147" t="str">
         <v>Nature</v>
       </c>
@@ -5744,6 +5939,9 @@
       <c r="B148" t="str">
         <v>Thunder is banging his drums way too loud again!</v>
       </c>
+      <c r="C148" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a rockstar-style dark grey thunder cloud with drumsticks, banging on tiny drums with an excited wild face"</v>
+      </c>
       <c r="D148" t="str">
         <v>Nature</v>
       </c>
@@ -5779,6 +5977,9 @@
       <c r="B149" t="str">
         <v>Wind is blowing out birthday candles that aren't even his!</v>
       </c>
+      <c r="C149" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a swirly light blue wind spirit with puffed cheeks blowing hard, a tiny birthday cake with candles going out"</v>
+      </c>
       <c r="D149" t="str">
         <v>Nature</v>
       </c>
@@ -5814,6 +6015,9 @@
       <c r="B150" t="str">
         <v>Eight is a snowman begging for warm hugs!</v>
       </c>
+      <c r="C150" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 8 dressed as a snowman with a tiny scarf and a top hat, both arms reaching out with a hopeful pleading face, having little cute feet"</v>
+      </c>
       <c r="D150" t="str">
         <v>Numbers</v>
       </c>
@@ -5821,7 +6025,7 @@
         <v>1</v>
       </c>
       <c r="F150" t="str">
-        <v>八</v>
+        <v>数字8</v>
       </c>
       <c r="G150" t="str">
         <v>bā</v>
@@ -5849,6 +6053,9 @@
       <c r="B151" t="str">
         <v>Five is a chubby little Santa with a big round belly!</v>
       </c>
+      <c r="C151" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 5 dressed as Santa with a red hat and white beard, its round bottom half looking like a big jolly tummy, having little cute feet"</v>
+      </c>
       <c r="D151" t="str">
         <v>Numbers</v>
       </c>
@@ -5856,7 +6063,7 @@
         <v>1</v>
       </c>
       <c r="F151" t="str">
-        <v>五</v>
+        <v>数字5</v>
       </c>
       <c r="G151" t="str">
         <v>wǔ</v>
@@ -5884,6 +6091,9 @@
       <c r="B152" t="str">
         <v>Four is a grumpy chair who hates being sat on!</v>
       </c>
+      <c r="C152" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 4 dressed as a wooden chair, with a grumpy annoyed face, tiny arms crossed"</v>
+      </c>
       <c r="D152" t="str">
         <v>Numbers</v>
       </c>
@@ -5891,7 +6101,7 @@
         <v>1</v>
       </c>
       <c r="F152" t="str">
-        <v>四</v>
+        <v>数字4</v>
       </c>
       <c r="G152" t="str">
         <v>sì</v>
@@ -5919,6 +6129,9 @@
       <c r="B153" t="str">
         <v>Nine is a smart professor with a giant brain.</v>
       </c>
+      <c r="C153" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 9 in professor-style with tiny glasses, its big round top looking like a giant brain, with a proud smart face"</v>
+      </c>
       <c r="D153" t="str">
         <v>Numbers</v>
       </c>
@@ -5926,7 +6139,7 @@
         <v>1</v>
       </c>
       <c r="F153" t="str">
-        <v>九</v>
+        <v>数字9</v>
       </c>
       <c r="G153" t="str">
         <v>jiǔ</v>
@@ -5954,6 +6167,9 @@
       <c r="B154" t="str">
         <v>One is a skinny pencil with a big eraser hat!</v>
       </c>
+      <c r="C154" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 1 dressed as a yellow pencil with a big pink eraser on top like a hat, with a cheerful face"</v>
+      </c>
       <c r="D154" t="str">
         <v>Numbers</v>
       </c>
@@ -5961,7 +6177,7 @@
         <v>1</v>
       </c>
       <c r="F154" t="str">
-        <v>一</v>
+        <v>数字1</v>
       </c>
       <c r="G154" t="str">
         <v>yī</v>
@@ -5989,6 +6205,9 @@
       <c r="B155" t="str">
         <v>Seven is a candy cane that never tastes like mint!</v>
       </c>
+      <c r="C155" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 7 dressed as a candy cane with red and white stripes, with a disappointed pouty face"</v>
+      </c>
       <c r="D155" t="str">
         <v>Numbers</v>
       </c>
@@ -5996,7 +6215,7 @@
         <v>1</v>
       </c>
       <c r="F155" t="str">
-        <v>七</v>
+        <v>数字7</v>
       </c>
       <c r="G155" t="str">
         <v>qī</v>
@@ -6024,6 +6243,9 @@
       <c r="B156" t="str">
         <v>Six is a little snail dragging her big round shell!</v>
       </c>
+      <c r="C156" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 6 dressed as a snail with tiny antennae, its round top looking like a big spiral shell, with a tired slow face"</v>
+      </c>
       <c r="D156" t="str">
         <v>Numbers</v>
       </c>
@@ -6031,7 +6253,7 @@
         <v>1</v>
       </c>
       <c r="F156" t="str">
-        <v>六</v>
+        <v>数字6</v>
       </c>
       <c r="G156" t="str">
         <v>liù</v>
@@ -6059,6 +6281,9 @@
       <c r="B157" t="str">
         <v>Ten is a baseball bat standing next to his fast little ball!</v>
       </c>
+      <c r="C157" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 1 dressed as a baseball bat with a sporty confident face, next to a number 0 dressed as a baseball with an excited face"</v>
+      </c>
       <c r="D157" t="str">
         <v>Numbers</v>
       </c>
@@ -6066,7 +6291,7 @@
         <v>1</v>
       </c>
       <c r="F157" t="str">
-        <v>十</v>
+        <v>数字10</v>
       </c>
       <c r="G157" t="str">
         <v>shí</v>
@@ -6094,6 +6319,9 @@
       <c r="B158" t="str">
         <v>Three is a chubby bumblebee too heavy to fly!</v>
       </c>
+      <c r="C158" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a chubby number 3 dressed as a bumblebee with tiny wings and yellow-black stripes, with a struggling exhausted face, having little cute feet"</v>
+      </c>
       <c r="D158" t="str">
         <v>Numbers</v>
       </c>
@@ -6101,7 +6329,7 @@
         <v>1</v>
       </c>
       <c r="F158" t="str">
-        <v>三</v>
+        <v>数字3</v>
       </c>
       <c r="G158" t="str">
         <v>sān</v>
@@ -6129,6 +6357,9 @@
       <c r="B159" t="str">
         <v>Two is a yellow ducky with a tiny orange beak!</v>
       </c>
+      <c r="C159" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 2 dressed as a yellow rubber ducky with a tiny orange beak, with a happy quacking face, having little cute feet"</v>
+      </c>
       <c r="D159" t="str">
         <v>Numbers</v>
       </c>
@@ -6136,7 +6367,7 @@
         <v>1</v>
       </c>
       <c r="F159" t="str">
-        <v>二</v>
+        <v>数字2</v>
       </c>
       <c r="G159" t="str">
         <v>èr</v>
@@ -6164,6 +6395,9 @@
       <c r="B160" t="str">
         <v>Zero is a giant donut with pink frosting on top!</v>
       </c>
+      <c r="C160" t="str">
+        <v>PlushStyle, plush style, white background, a super cute plush toy of "a number 0 dressed as a donut with pink frosting and colorful sprinkles, with a sweet happy face, having little cute feet"</v>
+      </c>
       <c r="D160" t="str">
         <v>Numbers</v>
       </c>
@@ -6171,7 +6405,7 @@
         <v>1</v>
       </c>
       <c r="F160" t="str">
-        <v>零</v>
+        <v>数字0</v>
       </c>
       <c r="G160" t="str">
         <v>líng</v>
@@ -6627,7 +6861,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B15"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -6643,87 +6877,119 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>vocab-food</v>
+        <v>vocab-animal</v>
       </c>
       <c r="B2" t="str">
-        <v>beef</v>
+        <v>pig</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>vocab-animal</v>
+        <v>vocab-adjective</v>
       </c>
       <c r="B3" t="str">
-        <v>bird</v>
+        <v>good</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>vocab-body</v>
+        <v>vocab-food</v>
       </c>
       <c r="B4" t="str">
-        <v>hand</v>
+        <v>mushroom</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>vocab-clothes</v>
+        <v>vocab-places</v>
       </c>
       <c r="B5" t="str">
-        <v>hat</v>
+        <v>airport</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>vocab-colors</v>
+        <v>vocab-body</v>
       </c>
       <c r="B6" t="str">
-        <v>pink</v>
+        <v>eye</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>vocab-places</v>
+        <v>vocab-clothes</v>
       </c>
       <c r="B7" t="str">
-        <v>bank</v>
+        <v>pants</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>oral-everyday</v>
+        <v>vocab-colors</v>
       </c>
       <c r="B8" t="str">
-        <v>cake</v>
+        <v>blue</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>oral-food</v>
+        <v>vocab-items</v>
       </c>
       <c r="B9" t="str">
-        <v>beef</v>
+        <v>computer</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>oral-emotions</v>
+        <v>vocab-nature</v>
       </c>
       <c r="B10" t="str">
-        <v>bear</v>
+        <v>rain</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>vocab-numbers</v>
+      </c>
+      <c r="B11" t="str">
+        <v>eight</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>oral-everyday</v>
+      </c>
+      <c r="B12" t="str">
+        <v>orange</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>oral-opinions</v>
       </c>
-      <c r="B11" t="str">
-        <v>elephant</v>
+      <c r="B13" t="str">
+        <v>cherry</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>oral-food</v>
+      </c>
+      <c r="B14" t="str">
+        <v>hungry</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>oral-emotions</v>
+      </c>
+      <c r="B15" t="str">
+        <v>durian</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>